<commit_message>
application-layer-protocol: add candidate release 2.0.0
</commit_message>
<xml_diff>
--- a/application-layer-protocol/application-layer-protocol.xlsx
+++ b/application-layer-protocol/application-layer-protocol.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scrocca\Desktop\cefriel-github\controlled-vocabularies\base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1ED3A00-24F1-48A1-931A-CE1E76F71BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8ADBAB-6813-4945-AEAC-A3ECE3B1E20D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2550" yWindow="2550" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,9 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -35,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="54">
   <si>
     <t>ConceptScheme URI</t>
   </si>
@@ -79,13 +82,22 @@
     <t>owl:versionIRI</t>
   </si>
   <si>
+    <t>owl:priorVersion</t>
+  </si>
+  <si>
+    <t>https://w3id.org/mobilitydcat-ap/application-layer-protocol/1.0.0</t>
+  </si>
+  <si>
     <t>dct:license</t>
   </si>
   <si>
     <t>https://creativecommons.org/licenses/by/4.0/</t>
   </si>
   <si>
-    <t>My comments (not parsed by the tool).</t>
+    <t>http://purl.org/ontology/bibo/status</t>
+  </si>
+  <si>
+    <t>Published Controlled Vocabulary</t>
   </si>
   <si>
     <t>URI</t>
@@ -97,7 +109,13 @@
     <t>skos:definition</t>
   </si>
   <si>
-    <t>skos:narrower</t>
+    <t>skos:broader</t>
+  </si>
+  <si>
+    <t>owl:deprecated^^xsd:boolean</t>
+  </si>
+  <si>
+    <t>dcterms:replacedBy</t>
   </si>
   <si>
     <t>skos:notation</t>
@@ -115,13 +133,31 @@
     <t>HTTP/HTTPS</t>
   </si>
   <si>
+    <t>https://w3id.org/mobilitydcat-ap/application-layer-protocol/http</t>
+  </si>
+  <si>
+    <t>SSE</t>
+  </si>
+  <si>
+    <t>Server-Sent Events (SSE)</t>
+  </si>
+  <si>
+    <t>REST</t>
+  </si>
+  <si>
+    <t>Long Polling</t>
+  </si>
+  <si>
+    <t>HTTP Long Polling</t>
+  </si>
+  <si>
     <t>SOAP</t>
   </si>
   <si>
-    <t>HTTP/HTTPS-SOAP</t>
-  </si>
-  <si>
-    <t>FTP</t>
+    <t>https://w3id.org/mobilitydcat-ap/application-layer-protocol/ftp</t>
+  </si>
+  <si>
+    <t>FTP/SFTP</t>
   </si>
   <si>
     <t>RSS</t>
@@ -136,26 +172,41 @@
     <t>gRPC</t>
   </si>
   <si>
+    <t>ZeroMQ</t>
+  </si>
+  <si>
     <t>Other</t>
   </si>
   <si>
-    <t>http://purl.org/ontology/bibo/status</t>
-  </si>
-  <si>
-    <t>owl:priorVersion</t>
-  </si>
-  <si>
-    <t>Published Controlled Vocabulary</t>
-  </si>
-  <si>
-    <t>1.0.0</t>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>Petr Bures (TamTam Research)</t>
+  </si>
+  <si>
+    <t>Simple Object Access Protocol (SOAP)</t>
+  </si>
+  <si>
+    <t>(Secure) File Transfer Protocol (FTP/SFTP)</t>
+  </si>
+  <si>
+    <t>Really Simple Syndication (RSS)</t>
+  </si>
+  <si>
+    <t>Hypertext Transfer Protocol (HTTP/HTTPS)</t>
+  </si>
+  <si>
+    <t>Advanced Message Queuing Protocol (AMQP)</t>
+  </si>
+  <si>
+    <t>gRPC Remote Procedure Call (gRPC)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -185,8 +236,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -196,6 +260,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -213,7 +295,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -230,6 +312,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
@@ -544,18 +653,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.5703125" customWidth="1"/>
-    <col min="2" max="2" width="67.5703125" customWidth="1"/>
-    <col min="3" max="3" width="52.5703125" customWidth="1"/>
-    <col min="4" max="4" width="45.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="35.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="30.42578125" customWidth="1"/>
+    <col min="1" max="1" width="71.85546875" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="48.140625" customWidth="1"/>
+    <col min="4" max="4" width="57.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="35" style="1" customWidth="1"/>
+    <col min="6" max="6" width="60.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="35.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="30.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -563,7 +674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
@@ -572,7 +683,7 @@
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -581,7 +692,7 @@
       </c>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -590,7 +701,7 @@
       </c>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -599,7 +710,7 @@
       </c>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
@@ -608,181 +719,316 @@
       </c>
       <c r="C6" s="1"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
+      <c r="B7" s="16" t="s">
+        <v>47</v>
+      </c>
       <c r="C7" s="1"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B9" t="s">
-        <v>37</v>
+      <c r="B9" s="13" t="s">
+        <v>46</v>
       </c>
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B10" t="str">
         <f>_xlfn.CONCAT(B1,"/",B9)</f>
-        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/1.0.0</v>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/2.0.0</v>
       </c>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="str">
+        <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B17)," ","-"),",",""))</f>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/ots2</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="12" t="str">
+        <f>A31</f>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/other</v>
+      </c>
+      <c r="G17" s="12"/>
+    </row>
+    <row r="18" spans="1:7" s="10" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="str">
+        <f t="shared" ref="A18:A31" si="0">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B18)," ","-"),",",""))</f>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/ocit</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" s="12" t="str">
+        <f>A31</f>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/other</v>
+      </c>
+      <c r="G18" s="12"/>
+    </row>
+    <row r="19" spans="1:7" s="10" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="str">
+        <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B19)," ","-"),",",""))</f>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/http-https</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" s="12" t="str">
+        <f>A20</f>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/http</v>
+      </c>
+      <c r="G19" s="12"/>
+    </row>
+    <row r="20" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+    </row>
+    <row r="21" spans="1:7" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/sse</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="15" t="str">
+        <f>A20</f>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/http</v>
+      </c>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+    </row>
+    <row r="22" spans="1:7" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/rest</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="15" t="str">
+        <f>A20</f>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/http</v>
+      </c>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+    </row>
+    <row r="23" spans="1:7" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/long-polling</v>
+      </c>
+      <c r="B23" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="1"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="1"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C23" s="14" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" t="str">
-        <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B18)," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/ots2</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" t="str">
-        <f t="shared" ref="A19:A27" si="0">_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B19)," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/ocit</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="str">
-        <f>_xlfn.CONCAT($B$1,"/",SUBSTITUTE(SUBSTITUTE(LOWER(B20)," ","-"),",",""))</f>
-        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/http-https</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="str">
+      <c r="D23" s="15" t="str">
+        <f>A20</f>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/http</v>
+      </c>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/soap</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="str">
-        <f t="shared" si="0"/>
-        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/ftp</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="str">
+      <c r="B24" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D24" s="18"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/rss</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="str">
+      <c r="B26" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/amqp</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="str">
+      <c r="B27" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/mqtt</v>
       </c>
-      <c r="B25" s="6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="str">
+      <c r="B28" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/grpc</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="str">
+      <c r="B29" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/zeromq</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="str">
         <f t="shared" si="0"/>
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/other</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B28" s="6"/>
+      <c r="B31" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -807,12 +1053,10 @@
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <TaxCatchAll xmlns="4ea66b1c-fa60-4493-a86c-b420df37761a" xsi:nil="true"/>
-    <Date_x002f_Heure xmlns="322c47a9-7cf9-4f39-ba36-4bf679c08fb0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="322c47a9-7cf9-4f39-ba36-4bf679c08fb0">
+    <TaxCatchAll xmlns="13e36eaf-61a1-47aa-b343-0f7d626aa9a0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
-    <note xmlns="322c47a9-7cf9-4f39-ba36-4bf679c08fb0" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
@@ -827,34 +1071,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100156B981FAAFB4349A28B03AB4EEECF9F" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1e7c9bb6974a57a0073a8d48fc3b6089">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4ea66b1c-fa60-4493-a86c-b420df37761a" xmlns:ns3="322c47a9-7cf9-4f39-ba36-4bf679c08fb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d5753863158ce54f5fdf0d8971fe3971" ns2:_="" ns3:_="">
-    <xsd:import namespace="4ea66b1c-fa60-4493-a86c-b420df37761a"/>
-    <xsd:import namespace="322c47a9-7cf9-4f39-ba36-4bf679c08fb0"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006748505E66128D48AAED90CD5CD3616F" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b912ec8155dd4e933917767331a7e7b9">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa" xmlns:ns3="13e36eaf-61a1-47aa-b343-0f7d626aa9a0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f994fb40b965d01e7e08c4f92ceb61cd" ns2:_="" ns3:_="">
+    <xsd:import namespace="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa"/>
+    <xsd:import namespace="13e36eaf-61a1-47aa-b343-0f7d626aa9a0"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element name="documentManagement">
             <xsd:complexType>
               <xsd:all>
-                <xsd:element ref="ns2:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns2:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns3:note" minOccurs="0"/>
-                <xsd:element ref="ns3:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns3:Date_x002f_Heure" minOccurs="0"/>
-                <xsd:element ref="ns3:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -862,36 +1099,68 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="4ea66b1c-fa60-4493-a86c-b420df37761a" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="8" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="84381483-150a-4726-b180-307f5f59d12b" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="9" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="23" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{517dfd69-ad1a-4b80-a735-177bb10dea14}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="4ea66b1c-fa60-4493-a86c-b420df37761a">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="13e36eaf-61a1-47aa-b343-0f7d626aa9a0" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{4c7b0293-1299-401f-a92e-ea8ec6326420}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="13e36eaf-61a1-47aa-b343-0f7d626aa9a0">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -901,93 +1170,6 @@
           </xsd:extension>
         </xsd:complexContent>
       </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="322c47a9-7cf9-4f39-ba36-4bf679c08fb0" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="10" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="13" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="17" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="18" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="note" ma:index="20" nillable="true" ma:displayName="note" ma:format="Dropdown" ma:internalName="note">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="22" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="84381483-150a-4726-b180-307f5f59d12b" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="24" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Date_x002f_Heure" ma:index="25" nillable="true" ma:displayName="Date/Heure" ma:format="DateTime" ma:internalName="Date_x002f_Heure">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:DateTime"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="26" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -1094,8 +1276,8 @@
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4ea66b1c-fa60-4493-a86c-b420df37761a"/>
-    <ds:schemaRef ds:uri="322c47a9-7cf9-4f39-ba36-4bf679c08fb0"/>
+    <ds:schemaRef ds:uri="13e36eaf-61a1-47aa-b343-0f7d626aa9a0"/>
+    <ds:schemaRef ds:uri="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1109,14 +1291,14 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60AB3605-D74C-42B6-A2DD-9EBC41B913EF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37572B91-55AC-4C8A-8FA1-60C7F6647852}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
     <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="4ea66b1c-fa60-4493-a86c-b420df37761a"/>
-    <ds:schemaRef ds:uri="322c47a9-7cf9-4f39-ba36-4bf679c08fb0"/>
+    <ds:schemaRef ds:uri="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa"/>
+    <ds:schemaRef ds:uri="13e36eaf-61a1-47aa-b343-0f7d626aa9a0"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>

</xml_diff>

<commit_message>
application-layer-protocol: fix candidate release 2.0.0
</commit_message>
<xml_diff>
--- a/application-layer-protocol/application-layer-protocol.xlsx
+++ b/application-layer-protocol/application-layer-protocol.xlsx
@@ -8,14 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scrocca\Desktop\cefriel-github\controlled-vocabularies\base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8ADBAB-6813-4945-AEAC-A3ECE3B1E20D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B67CCA69-F0DD-47D1-B5C0-116682239A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
-    <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
-    <sheet name="Feuil3" sheetId="3" r:id="rId3"/>
+    <sheet name="Vocabulary" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -97,9 +95,6 @@
     <t>http://purl.org/ontology/bibo/status</t>
   </si>
   <si>
-    <t>Published Controlled Vocabulary</t>
-  </si>
-  <si>
     <t>URI</t>
   </si>
   <si>
@@ -187,9 +182,6 @@
     <t>Simple Object Access Protocol (SOAP)</t>
   </si>
   <si>
-    <t>(Secure) File Transfer Protocol (FTP/SFTP)</t>
-  </si>
-  <si>
     <t>Really Simple Syndication (RSS)</t>
   </si>
   <si>
@@ -200,6 +192,12 @@
   </si>
   <si>
     <t>gRPC Remote Procedure Call (gRPC)</t>
+  </si>
+  <si>
+    <t>Draft Controlled Vocabulary</t>
+  </si>
+  <si>
+    <t>File Transfer Protocol (FTP/SFTP)</t>
   </si>
 </sst>
 </file>
@@ -295,7 +293,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -335,9 +333,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -643,15 +638,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G32"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -724,7 +710,7 @@
         <v>11</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C7" s="1"/>
     </row>
@@ -739,7 +725,7 @@
         <v>12</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9" s="1"/>
     </row>
@@ -776,30 +762,30 @@
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="10" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -808,7 +794,7 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/ots2</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="12" t="b">
@@ -826,7 +812,7 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/ocit</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="12" t="b">
@@ -844,10 +830,10 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/http-https</v>
       </c>
       <c r="B19" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="11" t="s">
         <v>29</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>30</v>
       </c>
       <c r="D19" s="12"/>
       <c r="E19" s="12" t="b">
@@ -861,13 +847,13 @@
     </row>
     <row r="20" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D20" s="15"/>
       <c r="E20" s="15"/>
@@ -880,10 +866,10 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/sse</v>
       </c>
       <c r="B21" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="14" t="s">
         <v>32</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>33</v>
       </c>
       <c r="D21" s="15" t="str">
         <f>A20</f>
@@ -899,10 +885,10 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/rest</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D22" s="15" t="str">
         <f>A20</f>
@@ -918,10 +904,10 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/long-polling</v>
       </c>
       <c r="B23" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C23" s="14" t="s">
         <v>35</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>36</v>
       </c>
       <c r="D23" s="15" t="str">
         <f>A20</f>
@@ -937,22 +923,21 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/soap</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="D24" s="18"/>
+        <v>47</v>
+      </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="8" t="s">
-        <v>39</v>
-      </c>
       <c r="C25" s="9" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -961,10 +946,10 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/rss</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,10 +958,10 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/amqp</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -985,10 +970,10 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/mqtt</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -997,10 +982,10 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/grpc</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1009,10 +994,10 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/zeromq</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1021,10 +1006,10 @@
         <v>https://w3id.org/mobilitydcat-ap/application-layer-protocol/other</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1038,15 +1023,6 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1062,15 +1038,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006748505E66128D48AAED90CD5CD3616F" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b912ec8155dd4e933917767331a7e7b9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa" xmlns:ns3="13e36eaf-61a1-47aa-b343-0f7d626aa9a0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f994fb40b965d01e7e08c4f92ceb61cd" ns2:_="" ns3:_="">
     <xsd:import namespace="c386cf2f-2f8b-4d8e-84b2-f14abf7317aa"/>
@@ -1271,6 +1238,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DC6AC960-8266-4EB4-8874-7C8BE96E25EB}">
   <ds:schemaRefs>
@@ -1283,14 +1259,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354E852E-38F4-443F-ABCC-E4BE2043727A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37572B91-55AC-4C8A-8FA1-60C7F6647852}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1307,4 +1275,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354E852E-38F4-443F-ABCC-E4BE2043727A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>